<commit_message>
Tweaks for final analysis
</commit_message>
<xml_diff>
--- a/working/CrizerPFAS/CrizerChemIDs-Feb2024.xlsx
+++ b/working/CrizerPFAS/CrizerChemIDs-Feb2024.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jwambaug\git\invitrotkstats\working\CrizerPFAS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EA9B80C-3841-4DFA-B5C1-3E973B99AEB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC5E6FCB-BE9E-4C45-85CB-AEFB851445AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1790" yWindow="940" windowWidth="13310" windowHeight="8970" xr2:uid="{819F4BB0-2119-468F-947F-0171544AB1A3}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{819F4BB0-2119-468F-947F-0171544AB1A3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>